<commit_message>
UI/UX reviewed to fit original need + modification of back end to import InputData .csv files and handle ExcelParameters files in constraints
</commit_message>
<xml_diff>
--- a/nw_allocation_tool/data/ExcelParameters/CoverageperABCperChannel.xlsx
+++ b/nw_allocation_tool/data/ExcelParameters/CoverageperABCperChannel.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://loreal-my.sharepoint.com/personal/nils_levillain_loreal_com/Documents/Desktop/Python/WindSurf/Test/ExcelParameters/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://loreal-my.sharepoint.com/personal/nils_levillain_loreal_com/Documents/Desktop/Python/No Waste Allocation Tool/nw_allocation_tool/data/ExcelParameters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{0AA7584F-D85B-436B-ABF0-9030EC79EE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65C82F4E-D5C0-47FE-9920-97530CBC929B}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{0AA7584F-D85B-436B-ABF0-9030EC79EE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30271F20-C90C-4193-9FAE-D423D1B2EE9D}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{18B4B8A2-C4B4-4780-A18C-FFEAEF7D9308}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{18B4B8A2-C4B4-4780-A18C-FFEAEF7D9308}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -254,23 +254,23 @@
       </border>
     </dxf>
     <dxf>
-      <border>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
+      <border>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -308,7 +308,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6DFE0357-6CD0-452F-9AAE-687E41C817B6}" name="Tableau5" displayName="Tableau5" ref="A1:C7" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="4" tableBorderDxfId="5" totalsRowBorderDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6DFE0357-6CD0-452F-9AAE-687E41C817B6}" name="Tableau5" displayName="Tableau5" ref="A1:C7" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="5" tableBorderDxfId="4" totalsRowBorderDxfId="3">
   <autoFilter ref="A1:C7" xr:uid="{6DFE0357-6CD0-452F-9AAE-687E41C817B6}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{2479C95F-9E31-465B-AEB8-0D7770B48D35}" name="Channel" dataDxfId="2"/>
@@ -638,6 +638,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F069EFA-C002-4A06-9C6E-F7079E647166}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.453125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">

</xml_diff>